<commit_message>
Fix cross-platform validation and synchronize review metadata
</commit_message>
<xml_diff>
--- a/precision_annotations/precision_annotations.xlsx
+++ b/precision_annotations/precision_annotations.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R9422fc57897941b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re472d593d9f34413"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="R45368249904c4ad2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Matrix" sheetId="4" r:id="R429f405a67ea4b4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Chain" sheetId="5" r:id="Re590d395cbcf4bbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artifacts" sheetId="6" r:id="R2e6ea1096a264c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="7" r:id="Re1d9ac49cf154e1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R27efe41fb3d0435c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re8deaaf203e746a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="R8ece2e01146e4ba9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Matrix" sheetId="4" r:id="R01bd99589c8a411f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Chain" sheetId="5" r:id="R1e4fc259e1864205"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artifacts" sheetId="6" r:id="R775e679cc2aa4b53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="7" r:id="Rd18be499203148c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2883,16 +2883,16 @@
         <x:v>handover</x:v>
       </x:c>
       <x:c r="F9" s="14" t="str">
-        <x:v>ContactHandover: Contact-Aware Handovers with Dexterous Hands</x:v>
+        <x:v>ContactHandover: Contact-Guided Robot-to-Human Object Handover</x:v>
       </x:c>
       <x:c r="G9" s="14" t="str">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="H9" s="14" t="str">
-        <x:v>preprint</x:v>
+        <x:v>IROS 2024</x:v>
       </x:c>
       <x:c r="I9" s="14" t="str">
-        <x:v>https://arxiv.org/abs/2404.01402</x:v>
+        <x:v>https://doi.org/10.1109/IROS58592.2024.10801777</x:v>
       </x:c>
       <x:c r="J9" s="14" t="str">
         <x:v>referenced/01_bimanual_handover/2024_ContactHandover.pdf</x:v>
@@ -8642,7 +8642,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R162866023cd7418a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R453d06916af04f30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9940,7 +9940,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04c47cb8cf2d4d74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9929b0c8999f4b43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10862,7 +10862,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra075230acec34577"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5e928ee1c444c17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11197,7 +11197,7 @@
         <x:v>ContactHandover</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
-        <x:v>preprint</x:v>
+        <x:v>IROS 2024</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
         <x:v>NR</x:v>
@@ -12066,7 +12066,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8acd1ff532740c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb819ea6254047aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>